<commit_message>
fix(engine): Renditen als Jahresertrag — gleiche Logik wie LV
Fachliche Entscheidung: Eingegebene Renditen sind Jahresertraege ohne
unterjaehrigen Zinseszins (7 % − 1,5 % Kosten = 5,5 % p.a.). Drift jetzt
ln(1 + r) statt r → Durchschnitt der Jahresrenditen genau r, wie bei der
fondsgebundenen LV. Vorher: exp(r) − 1 = 5,65 % p.a.

Referenzen bewusst neu eingefroren: Erfolgsquoten 0–3 pp niedriger,
historischer Backtest unveraendert. Excel-Gegenrechnung auf
Jahresrendite = Brutto − Kosten umgestellt (Abweichung weiter 0,00 EUR).
depositTax.test: erwarteter Effektivzins = Eingabe.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Gegenrechnung_Referenzfaelle.xlsx
+++ b/docs/Gegenrechnung_Referenzfaelle.xlsx
@@ -52,13 +52,13 @@
     <t>Alle Fälle ohne Schwankung (Volatilität 0) und ohne Umschichtung, damit jede Zahl eindeutig nachrechenbar ist.</t>
   </si>
   <si>
-    <t>Zur Prüfung vorgelegte Modellannahme</t>
+    <t>Modellannahme</t>
   </si>
   <si>
     <t>Renditeformel</t>
   </si>
   <si>
-    <t>Die App verzinst stetig: Jahresrendite = EXP(Brutto − Kosten) − 1. Aus 7,0 % Brutto − 1,5 % Kosten werden so 5,65 % statt 5,50 %. Bei Schwankung ist der Mittelwert der Jahresrenditen ebenfalls EXP(Brutto − Kosten) − 1. Die fondsgebundene LV rechnet dagegen mit ln(1 + Ertragserwartung), trifft also die Eingabe genau. Bitte fachlich entscheiden, welche Lesart der eingegebenen Renditen gilt.</t>
+    <t>Eingegebene Renditen sind Jahreserträge: Jahresrendite = Brutto − Kosten (7,0 % − 1,5 % = 5,50 % p.a.). Zinseszins entsteht über die Jahre. Bei Schwankung ist der Durchschnitt der Jahresrenditen genau dieser Wert; der typische (mittlere) Verlauf liegt wegen der Schwankung darunter. Wertpapier-Töpfe und fondsgebundene LV rechnen nach derselben Logik.</t>
   </si>
   <si>
     <t>Fall</t>
@@ -817,7 +817,7 @@
         <f>'Fall 1'!AL60</f>
       </c>
       <c r="C13" s="5">
-        <v>115238.78850561776</v>
+        <v>97758.12028474794</v>
       </c>
       <c r="D13" s="6">
         <f>B13-C13</f>
@@ -831,7 +831,7 @@
         <f>'Fall 2'!AL61</f>
       </c>
       <c r="C14" s="5">
-        <v>187867.951225735</v>
+        <v>167645.08566528815</v>
       </c>
       <c r="D14" s="6">
         <f>B14-C14</f>
@@ -845,7 +845,7 @@
         <f>'Fall 3'!AL60</f>
       </c>
       <c r="C15" s="5">
-        <v>322638.7281853139</v>
+        <v>310590.049736207</v>
       </c>
       <c r="D15" s="6">
         <f>B15-C15</f>
@@ -1199,13 +1199,13 @@
         <f>$B$4</f>
       </c>
       <c r="H31" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I31" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J31" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K31" s="4">
         <f>D31*H31</f>
@@ -1292,7 +1292,7 @@
         <f>AH31+AI31+AJ31</f>
       </c>
       <c r="AM31" s="5">
-        <v>321198.8050311599</v>
+        <v>320995.125</v>
       </c>
       <c r="AN31" s="6">
         <f>AL31-AM31</f>
@@ -1321,13 +1321,13 @@
         <f>AK31</f>
       </c>
       <c r="H32" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I32" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J32" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K32" s="4">
         <f>D32*H32</f>
@@ -1414,7 +1414,7 @@
         <f>AH32+AI32+AJ32</f>
       </c>
       <c r="AM32" s="5">
-        <v>343394.32545903046</v>
+        <v>342962.3653282145</v>
       </c>
       <c r="AN32" s="6">
         <f>AL32-AM32</f>
@@ -1443,13 +1443,13 @@
         <f>AK32</f>
       </c>
       <c r="H33" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I33" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J33" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K33" s="4">
         <f>D33*H33</f>
@@ -1536,7 +1536,7 @@
         <f>AH33+AI33+AJ33</f>
       </c>
       <c r="AM33" s="5">
-        <v>366629.54927765625</v>
+        <v>365942.83524932107</v>
       </c>
       <c r="AN33" s="6">
         <f>AL33-AM33</f>
@@ -1565,13 +1565,13 @@
         <f>AK33</f>
       </c>
       <c r="H34" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I34" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J34" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K34" s="4">
         <f>D34*H34</f>
@@ -1658,7 +1658,7 @@
         <f>AH34+AI34+AJ34</f>
       </c>
       <c r="AM34" s="5">
-        <v>390949.2678921892</v>
+        <v>389979.3354292249</v>
       </c>
       <c r="AN34" s="6">
         <f>AL34-AM34</f>
@@ -1687,13 +1687,13 @@
         <f>AK34</f>
       </c>
       <c r="H35" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I35" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J35" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K35" s="4">
         <f>D35*H35</f>
@@ -1780,7 +1780,7 @@
         <f>AH35+AI35+AJ35</f>
       </c>
       <c r="AM35" s="5">
-        <v>416400.1512149429</v>
+        <v>415116.42146316136</v>
       </c>
       <c r="AN35" s="6">
         <f>AL35-AM35</f>
@@ -1809,13 +1809,13 @@
         <f>AK35</f>
       </c>
       <c r="H36" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I36" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J36" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K36" s="4">
         <f>D36*H36</f>
@@ -1902,7 +1902,7 @@
         <f>AH36+AI36+AJ36</f>
       </c>
       <c r="AM36" s="5">
-        <v>443030.8258465668</v>
+        <v>441400.475148458</v>
       </c>
       <c r="AN36" s="6">
         <f>AL36-AM36</f>
@@ -1931,13 +1931,13 @@
         <f>AK36</f>
       </c>
       <c r="H37" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I37" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J37" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K37" s="4">
         <f>D37*H37</f>
@@ -2024,7 +2024,7 @@
         <f>AH37+AI37+AJ37</f>
       </c>
       <c r="AM37" s="5">
-        <v>470891.9564725958</v>
+        <v>468879.7786149106</v>
       </c>
       <c r="AN37" s="6">
         <f>AL37-AM37</f>
@@ -2053,13 +2053,13 @@
         <f>AK37</f>
       </c>
       <c r="H38" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I38" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J38" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K38" s="4">
         <f>D38*H38</f>
@@ -2146,7 +2146,7 @@
         <f>AH38+AI38+AJ38</f>
       </c>
       <c r="AM38" s="5">
-        <v>500036.3306103863</v>
+        <v>497604.5914297255</v>
       </c>
       <c r="AN38" s="6">
         <f>AL38-AM38</f>
@@ -2175,13 +2175,13 @@
         <f>AK38</f>
       </c>
       <c r="H39" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I39" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J39" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K39" s="4">
         <f>D39*H39</f>
@@ -2268,7 +2268,7 @@
         <f>AH39+AI39+AJ39</f>
       </c>
       <c r="AM39" s="5">
-        <v>530518.9468465329</v>
+        <v>527627.2307982484</v>
       </c>
       <c r="AN39" s="6">
         <f>AL39-AM39</f>
@@ -2297,13 +2297,13 @@
         <f>AK39</f>
       </c>
       <c r="H40" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I40" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J40" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K40" s="4">
         <f>D40*H40</f>
@@ -2390,7 +2390,7 @@
         <f>AH40+AI40+AJ40</f>
       </c>
       <c r="AM40" s="5">
-        <v>562397.1067102428</v>
+        <v>559002.1549862225</v>
       </c>
       <c r="AN40" s="6">
         <f>AL40-AM40</f>
@@ -2419,13 +2419,13 @@
         <f>AK40</f>
       </c>
       <c r="H41" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I41" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J41" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K41" s="4">
         <f>D41*H41</f>
@@ -2512,7 +2512,7 @@
         <f>AH41+AI41+AJ41</f>
       </c>
       <c r="AM41" s="5">
-        <v>551644.3986317093</v>
+        <v>547699.9383919688</v>
       </c>
       <c r="AN41" s="6">
         <f>AL41-AM41</f>
@@ -2541,13 +2541,13 @@
         <f>AK41</f>
       </c>
       <c r="H42" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I42" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J42" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K42" s="4">
         <f>D42*H42</f>
@@ -2634,7 +2634,7 @@
         <f>AH42+AI42+AJ42</f>
       </c>
       <c r="AM42" s="5">
-        <v>540511.8715316398</v>
+        <v>535981.9491965759</v>
       </c>
       <c r="AN42" s="6">
         <f>AL42-AM42</f>
@@ -2663,13 +2663,13 @@
         <f>AK42</f>
       </c>
       <c r="H43" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I43" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J43" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K43" s="4">
         <f>D43*H43</f>
@@ -2756,7 +2756,7 @@
         <f>AH43+AI43+AJ43</f>
       </c>
       <c r="AM43" s="5">
-        <v>528988.3937595906</v>
+        <v>523835.39762286743</v>
       </c>
       <c r="AN43" s="6">
         <f>AL43-AM43</f>
@@ -2785,13 +2785,13 @@
         <f>AK43</f>
       </c>
       <c r="H44" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I44" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J44" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K44" s="4">
         <f>D44*H44</f>
@@ -2878,7 +2878,7 @@
         <f>AH44+AI44+AJ44</f>
       </c>
       <c r="AM44" s="5">
-        <v>516598.7226950218</v>
+        <v>510801.7431827362</v>
       </c>
       <c r="AN44" s="6">
         <f>AL44-AM44</f>
@@ -2907,13 +2907,13 @@
         <f>AK44</f>
       </c>
       <c r="H45" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I45" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J45" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K45" s="4">
         <f>D45*H45</f>
@@ -3000,7 +3000,7 @@
         <f>AH45+AI45+AJ45</f>
       </c>
       <c r="AM45" s="5">
-        <v>503080.5530673288</v>
+        <v>496624.03738812776</v>
       </c>
       <c r="AN45" s="6">
         <f>AL45-AM45</f>
@@ -3029,13 +3029,13 @@
         <f>AK45</f>
       </c>
       <c r="H46" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I46" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J46" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K46" s="4">
         <f>D46*H46</f>
@@ -3122,7 +3122,7 @@
         <f>AH46+AI46+AJ46</f>
       </c>
       <c r="AM46" s="5">
-        <v>488372.54640286864</v>
+        <v>481241.59379481326</v>
       </c>
       <c r="AN46" s="6">
         <f>AL46-AM46</f>
@@ -3151,13 +3151,13 @@
         <f>AK46</f>
       </c>
       <c r="H47" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I47" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J47" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K47" s="4">
         <f>D47*H47</f>
@@ -3244,7 +3244,7 @@
         <f>AH47+AI47+AJ47</f>
       </c>
       <c r="AM47" s="5">
-        <v>472410.40677849733</v>
+        <v>464590.86933323974</v>
       </c>
       <c r="AN47" s="6">
         <f>AL47-AM47</f>
@@ -3273,13 +3273,13 @@
         <f>AK47</f>
       </c>
       <c r="H48" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I48" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J48" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K48" s="4">
         <f>D48*H48</f>
@@ -3366,7 +3366,7 @@
         <f>AH48+AI48+AJ48</f>
       </c>
       <c r="AM48" s="5">
-        <v>455126.74756589683</v>
+        <v>446605.33847824426</v>
       </c>
       <c r="AN48" s="6">
         <f>AL48-AM48</f>
@@ -3395,13 +3395,13 @@
         <f>AK48</f>
       </c>
       <c r="H49" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I49" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J49" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K49" s="4">
         <f>D49*H49</f>
@@ -3488,7 +3488,7 @@
         <f>AH49+AI49+AJ49</f>
       </c>
       <c r="AM49" s="5">
-        <v>436450.9524426925</v>
+        <v>427215.3621249582</v>
       </c>
       <c r="AN49" s="6">
         <f>AL49-AM49</f>
@@ -3517,13 +3517,13 @@
         <f>AK49</f>
       </c>
       <c r="H50" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I50" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J50" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K50" s="4">
         <f>D50*H50</f>
@@ -3610,7 +3610,7 @@
         <f>AH50+AI50+AJ50</f>
       </c>
       <c r="AM50" s="5">
-        <v>416309.0304285393</v>
+        <v>406348.0509530125</v>
       </c>
       <c r="AN50" s="6">
         <f>AL50-AM50</f>
@@ -3639,13 +3639,13 @@
         <f>AK50</f>
       </c>
       <c r="H51" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I51" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J51" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K51" s="4">
         <f>D51*H51</f>
@@ -3732,7 +3732,7 @@
         <f>AH51+AI51+AJ51</f>
       </c>
       <c r="AM51" s="5">
-        <v>394623.4646942053</v>
+        <v>383927.1230522367</v>
       </c>
       <c r="AN51" s="6">
         <f>AL51-AM51</f>
@@ -3761,13 +3761,13 @@
         <f>AK51</f>
       </c>
       <c r="H52" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I52" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J52" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K52" s="4">
         <f>D52*H52</f>
@@ -3854,7 +3854,7 @@
         <f>AH52+AI52+AJ52</f>
       </c>
       <c r="AM52" s="5">
-        <v>371313.054881096</v>
+        <v>359872.7555737726</v>
       </c>
       <c r="AN52" s="6">
         <f>AL52-AM52</f>
@@ -3883,13 +3883,13 @@
         <f>AK52</f>
       </c>
       <c r="H53" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I53" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J53" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K53" s="4">
         <f>D53*H53</f>
@@ -3976,7 +3976,7 @@
         <f>AH53+AI53+AJ53</f>
       </c>
       <c r="AM53" s="5">
-        <v>346292.7526576541</v>
+        <v>334101.4301608702</v>
       </c>
       <c r="AN53" s="6">
         <f>AL53-AM53</f>
@@ -4005,13 +4005,13 @@
         <f>AK53</f>
       </c>
       <c r="H54" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I54" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J54" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K54" s="4">
         <f>D54*H54</f>
@@ -4098,7 +4098,7 @@
         <f>AH54+AI54+AJ54</f>
       </c>
       <c r="AM54" s="5">
-        <v>319473.49022759794</v>
+        <v>306525.7719035954</v>
       </c>
       <c r="AN54" s="6">
         <f>AL54-AM54</f>
@@ -4127,13 +4127,13 @@
         <f>AK54</f>
       </c>
       <c r="H55" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I55" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J55" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K55" s="4">
         <f>D55*H55</f>
@@ -4220,7 +4220,7 @@
         <f>AH55+AI55+AJ55</f>
       </c>
       <c r="AM55" s="5">
-        <v>290762.00149301504</v>
+        <v>277054.3815512325</v>
       </c>
       <c r="AN55" s="6">
         <f>AL55-AM55</f>
@@ -4249,13 +4249,13 @@
         <f>AK55</f>
       </c>
       <c r="H56" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I56" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J56" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K56" s="4">
         <f>D56*H56</f>
@@ -4342,7 +4342,7 @@
         <f>AH56+AI56+AJ56</f>
       </c>
       <c r="AM56" s="5">
-        <v>260060.63556289324</v>
+        <v>245591.6607053005</v>
       </c>
       <c r="AN56" s="6">
         <f>AL56-AM56</f>
@@ -4371,13 +4371,13 @@
         <f>AK56</f>
       </c>
       <c r="H57" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I57" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J57" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K57" s="4">
         <f>D57*H57</f>
@@ -4464,7 +4464,7 @@
         <f>AH57+AI57+AJ57</f>
       </c>
       <c r="AM57" s="5">
-        <v>227267.1622847161</v>
+        <v>212037.62970479793</v>
       </c>
       <c r="AN57" s="6">
         <f>AL57-AM57</f>
@@ -4493,13 +4493,13 @@
         <f>AK57</f>
       </c>
       <c r="H58" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I58" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J58" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K58" s="4">
         <f>D58*H58</f>
@@ -4586,7 +4586,7 @@
         <f>AH58+AI58+AJ58</f>
       </c>
       <c r="AM58" s="5">
-        <v>192274.5694632663</v>
+        <v>176287.73790352975</v>
       </c>
       <c r="AN58" s="6">
         <f>AL58-AM58</f>
@@ -4615,13 +4615,13 @@
         <f>AK58</f>
       </c>
       <c r="H59" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I59" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J59" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K59" s="4">
         <f>D59*H59</f>
@@ -4708,7 +4708,7 @@
         <f>AH59+AI59+AJ59</f>
       </c>
       <c r="AM59" s="5">
-        <v>154970.85141673568</v>
+        <v>138232.66602714016</v>
       </c>
       <c r="AN59" s="6">
         <f>AL59-AM59</f>
@@ -4737,13 +4737,13 @@
         <f>AK59</f>
       </c>
       <c r="H60" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I60" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J60" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K60" s="4">
         <f>D60*H60</f>
@@ -4830,7 +4830,7 @@
         <f>AH60+AI60+AJ60</f>
       </c>
       <c r="AM60" s="5">
-        <v>115238.78850561776</v>
+        <v>97758.12028474794</v>
       </c>
       <c r="AN60" s="6">
         <f>AL60-AM60</f>
@@ -5196,13 +5196,13 @@
         <f>$B$4</f>
       </c>
       <c r="H32" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I32" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J32" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K32" s="4">
         <f>D32*H32</f>
@@ -5289,7 +5289,7 @@
         <f>AH32+AI32+AJ32</f>
       </c>
       <c r="AM32" s="5">
-        <v>260247.98640993336</v>
+        <v>259968.75</v>
       </c>
       <c r="AN32" s="6">
         <f>AL32-AM32</f>
@@ -5318,13 +5318,13 @@
         <f>AK32</f>
       </c>
       <c r="H33" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I33" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J33" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K33" s="4">
         <f>D33*H33</f>
@@ -5411,7 +5411,7 @@
         <f>AH33+AI33+AJ33</f>
       </c>
       <c r="AM33" s="5">
-        <v>270916.0577216994</v>
+        <v>270335.00390625</v>
       </c>
       <c r="AN33" s="6">
         <f>AL33-AM33</f>
@@ -5440,13 +5440,13 @@
         <f>AK33</f>
       </c>
       <c r="H34" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I34" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J34" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K34" s="4">
         <f>D34*H34</f>
@@ -5533,7 +5533,7 @@
         <f>AH34+AI34+AJ34</f>
       </c>
       <c r="AM34" s="5">
-        <v>282021.4340327582</v>
+        <v>281114.6121870117</v>
       </c>
       <c r="AN34" s="6">
         <f>AL34-AM34</f>
@@ -5562,13 +5562,13 @@
         <f>AK34</f>
       </c>
       <c r="H35" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I35" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J35" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K35" s="4">
         <f>D35*H35</f>
@@ -5655,7 +5655,7 @@
         <f>AH35+AI35+AJ35</f>
       </c>
       <c r="AM35" s="5">
-        <v>293582.0413258687</v>
+        <v>292324.05734796874</v>
       </c>
       <c r="AN35" s="6">
         <f>AL35-AM35</f>
@@ -5684,13 +5684,13 @@
         <f>AK35</f>
       </c>
       <c r="H36" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I36" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J36" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K36" s="4">
         <f>D36*H36</f>
@@ -5777,7 +5777,7 @@
         <f>AH36+AI36+AJ36</f>
       </c>
       <c r="AM36" s="5">
-        <v>305616.5404047007</v>
+        <v>303980.479134719</v>
       </c>
       <c r="AN36" s="6">
         <f>AL36-AM36</f>
@@ -5806,13 +5806,13 @@
         <f>AK36</f>
       </c>
       <c r="H37" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I37" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J37" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K37" s="4">
         <f>D37*H37</f>
@@ -5899,7 +5899,7 @@
         <f>AH37+AI37+AJ37</f>
       </c>
       <c r="AM37" s="5">
-        <v>348144.35701557354</v>
+        <v>346101.7007402159</v>
       </c>
       <c r="AN37" s="6">
         <f>AL37-AM37</f>
@@ -5928,13 +5928,13 @@
         <f>AK37</f>
       </c>
       <c r="H38" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I38" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J38" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K38" s="4">
         <f>D38*H38</f>
@@ -6021,7 +6021,7 @@
         <f>AH38+AI38+AJ38</f>
       </c>
       <c r="AM38" s="5">
-        <v>362415.4715731358</v>
+        <v>359902.506057232</v>
       </c>
       <c r="AN38" s="6">
         <f>AL38-AM38</f>
@@ -6050,13 +6050,13 @@
         <f>AK38</f>
       </c>
       <c r="H39" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I39" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J39" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K39" s="4">
         <f>D39*H39</f>
@@ -6143,7 +6143,7 @@
         <f>AH39+AI39+AJ39</f>
       </c>
       <c r="AM39" s="5">
-        <v>377271.58688286017</v>
+        <v>374253.6184862641</v>
       </c>
       <c r="AN39" s="6">
         <f>AL39-AM39</f>
@@ -6172,13 +6172,13 @@
         <f>AK39</f>
       </c>
       <c r="H40" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I40" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J40" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K40" s="4">
         <f>D40*H40</f>
@@ -6265,7 +6265,7 @@
         <f>AH40+AI40+AJ40</f>
       </c>
       <c r="AM40" s="5">
-        <v>392736.68326377834</v>
+        <v>389176.98152340384</v>
       </c>
       <c r="AN40" s="6">
         <f>AL40-AM40</f>
@@ -6294,13 +6294,13 @@
         <f>AK40</f>
       </c>
       <c r="H41" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I41" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J41" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K41" s="4">
         <f>D41*H41</f>
@@ -6387,7 +6387,7 @@
         <f>AH41+AI41+AJ41</f>
       </c>
       <c r="AM41" s="5">
-        <v>408835.7240348563</v>
+        <v>404695.41366164957</v>
       </c>
       <c r="AN41" s="6">
         <f>AL41-AM41</f>
@@ -6416,13 +6416,13 @@
         <f>AK41</f>
       </c>
       <c r="H42" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I42" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J42" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K42" s="4">
         <f>D42*H42</f>
@@ -6509,7 +6509,7 @@
         <f>AH42+AI42+AJ42</f>
       </c>
       <c r="AM42" s="5">
-        <v>407690.10576919117</v>
+        <v>402928.05324052484</v>
       </c>
       <c r="AN42" s="6">
         <f>AL42-AM42</f>
@@ -6538,13 +6538,13 @@
         <f>AK42</f>
       </c>
       <c r="H43" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I43" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J43" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K43" s="4">
         <f>D43*H43</f>
@@ -6631,7 +6631,7 @@
         <f>AH43+AI43+AJ43</f>
       </c>
       <c r="AM43" s="5">
-        <v>406139.4345810383</v>
+        <v>400732.1275217901</v>
       </c>
       <c r="AN43" s="6">
         <f>AL43-AM43</f>
@@ -6660,13 +6660,13 @@
         <f>AK43</f>
       </c>
       <c r="H44" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I44" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J44" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K44" s="4">
         <f>D44*H44</f>
@@ -6753,7 +6753,7 @@
         <f>AH44+AI44+AJ44</f>
       </c>
       <c r="AM44" s="5">
-        <v>404159.94472700165</v>
+        <v>398083.3856281868</v>
       </c>
       <c r="AN44" s="6">
         <f>AL44-AM44</f>
@@ -6782,13 +6782,13 @@
         <f>AK44</f>
       </c>
       <c r="H45" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I45" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J45" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K45" s="4">
         <f>D45*H45</f>
@@ -6875,7 +6875,7 @@
         <f>AH45+AI45+AJ45</f>
       </c>
       <c r="AM45" s="5">
-        <v>401726.75302290317</v>
+        <v>394956.4664420054</v>
       </c>
       <c r="AN45" s="6">
         <f>AL45-AM45</f>
@@ -6904,13 +6904,13 @@
         <f>AK45</f>
       </c>
       <c r="H46" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I46" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J46" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K46" s="4">
         <f>D46*H46</f>
@@ -6997,7 +6997,7 @@
         <f>AH46+AI46+AJ46</f>
       </c>
       <c r="AM46" s="5">
-        <v>398813.81017297716</v>
+        <v>391324.85146951285</v>
       </c>
       <c r="AN46" s="6">
         <f>AL46-AM46</f>
@@ -7026,13 +7026,13 @@
         <f>AK46</f>
       </c>
       <c r="H47" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I47" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J47" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K47" s="4">
         <f>D47*H47</f>
@@ -7119,7 +7119,7 @@
         <f>AH47+AI47+AJ47</f>
       </c>
       <c r="AM47" s="5">
-        <v>345393.85004665796</v>
+        <v>337160.8157685548</v>
       </c>
       <c r="AN47" s="6">
         <f>AL47-AM47</f>
@@ -7148,13 +7148,13 @@
         <f>AK47</f>
       </c>
       <c r="H48" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I48" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J48" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K48" s="4">
         <f>D48*H48</f>
@@ -7241,7 +7241,7 @@
         <f>AH48+AI48+AJ48</f>
       </c>
       <c r="AM48" s="5">
-        <v>339388.73953569785</v>
+        <v>330441.626860955</v>
       </c>
       <c r="AN48" s="6">
         <f>AL48-AM48</f>
@@ -7270,13 +7270,13 @@
         <f>AK48</f>
       </c>
       <c r="H49" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I49" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J49" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K49" s="4">
         <f>D49*H49</f>
@@ -7363,7 +7363,7 @@
         <f>AH49+AI49+AJ49</f>
       </c>
       <c r="AM49" s="5">
-        <v>332734.1983323845</v>
+        <v>323051.2407669372</v>
       </c>
       <c r="AN49" s="6">
         <f>AL49-AM49</f>
@@ -7392,13 +7392,13 @@
         <f>AK49</f>
       </c>
       <c r="H50" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I50" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J50" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K50" s="4">
         <f>D50*H50</f>
@@ -7485,7 +7485,7 @@
         <f>AH50+AI50+AJ50</f>
       </c>
       <c r="AM50" s="5">
-        <v>325395.53961850563</v>
+        <v>314954.8281081185</v>
       </c>
       <c r="AN50" s="6">
         <f>AL50-AM50</f>
@@ -7514,13 +7514,13 @@
         <f>AK50</f>
       </c>
       <c r="H51" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I51" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J51" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K51" s="4">
         <f>D51*H51</f>
@@ -7607,7 +7607,7 @@
         <f>AH51+AI51+AJ51</f>
       </c>
       <c r="AM51" s="5">
-        <v>317336.4933878708</v>
+        <v>306116.00937684136</v>
       </c>
       <c r="AN51" s="6">
         <f>AL51-AM51</f>
@@ -7636,13 +7636,13 @@
         <f>AK51</f>
       </c>
       <c r="H52" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I52" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J52" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K52" s="4">
         <f>D52*H52</f>
@@ -7729,7 +7729,7 @@
         <f>AH52+AI52+AJ52</f>
       </c>
       <c r="AM52" s="5">
-        <v>308519.1383221999</v>
+        <v>296496.7898986128</v>
       </c>
       <c r="AN52" s="6">
         <f>AL52-AM52</f>
@@ -7758,13 +7758,13 @@
         <f>AK52</f>
       </c>
       <c r="H53" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I53" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J53" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K53" s="4">
         <f>D53*H53</f>
@@ -7851,7 +7851,7 @@
         <f>AH53+AI53+AJ53</f>
       </c>
       <c r="AM53" s="5">
-        <v>298903.83080994827</v>
+        <v>286057.4921366473</v>
       </c>
       <c r="AN53" s="6">
         <f>AL53-AM53</f>
@@ -7880,13 +7880,13 @@
         <f>AK53</f>
       </c>
       <c r="H54" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I54" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J54" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K54" s="4">
         <f>D54*H54</f>
@@ -7973,7 +7973,7 @@
         <f>AH54+AI54+AJ54</f>
       </c>
       <c r="AM54" s="5">
-        <v>288449.1309896616</v>
+        <v>274756.68523123994</v>
       </c>
       <c r="AN54" s="6">
         <f>AL54-AM54</f>
@@ -8002,13 +8002,13 @@
         <f>AK54</f>
       </c>
       <c r="H55" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I55" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J55" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K55" s="4">
         <f>D55*H55</f>
@@ -8095,7 +8095,7 @@
         <f>AH55+AI55+AJ55</f>
       </c>
       <c r="AM55" s="5">
-        <v>277111.72569457494</v>
+        <v>262551.1116623924</v>
       </c>
       <c r="AN55" s="6">
         <f>AL55-AM55</f>
@@ -8124,13 +8124,13 @@
         <f>AK55</f>
       </c>
       <c r="H56" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I56" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J56" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K56" s="4">
         <f>D56*H56</f>
@@ -8217,7 +8217,7 @@
         <f>AH56+AI56+AJ56</f>
       </c>
       <c r="AM56" s="5">
-        <v>264846.34817008756</v>
+        <v>249395.61091963816</v>
       </c>
       <c r="AN56" s="6">
         <f>AL56-AM56</f>
@@ -8246,13 +8246,13 @@
         <f>AK56</f>
       </c>
       <c r="H57" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I57" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J57" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K57" s="4">
         <f>D57*H57</f>
@@ -8339,7 +8339,7 @@
         <f>AH57+AI57+AJ57</f>
       </c>
       <c r="AM57" s="5">
-        <v>251605.69443045973</v>
+        <v>235243.04005836073</v>
       </c>
       <c r="AN57" s="6">
         <f>AL57-AM57</f>
@@ -8368,13 +8368,13 @@
         <f>AK57</f>
       </c>
       <c r="H58" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I58" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J58" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K58" s="4">
         <f>D58*H58</f>
@@ -8461,7 +8461,7 @@
         <f>AH58+AI58+AJ58</f>
       </c>
       <c r="AM58" s="5">
-        <v>237340.33611556856</v>
+        <v>220044.1910170559</v>
       </c>
       <c r="AN58" s="6">
         <f>AL58-AM58</f>
@@ -8490,13 +8490,13 @@
         <f>AK58</f>
       </c>
       <c r="H59" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I59" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J59" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K59" s="4">
         <f>D59*H59</f>
@@ -8583,7 +8583,7 @@
         <f>AH59+AI59+AJ59</f>
       </c>
       <c r="AM59" s="5">
-        <v>221998.6297028294</v>
+        <v>203747.70456495645</v>
       </c>
       <c r="AN59" s="6">
         <f>AL59-AM59</f>
@@ -8612,13 +8612,13 @@
         <f>AK59</f>
       </c>
       <c r="H60" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I60" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J60" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K60" s="4">
         <f>D60*H60</f>
@@ -8705,7 +8705,7 @@
         <f>AH60+AI60+AJ60</f>
       </c>
       <c r="AM60" s="5">
-        <v>205526.62192342043</v>
+        <v>186299.98074420143</v>
       </c>
       <c r="AN60" s="6">
         <f>AL60-AM60</f>
@@ -8734,13 +8734,13 @@
         <f>AK60</f>
       </c>
       <c r="H61" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I61" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J61" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K61" s="4">
         <f>D61*H61</f>
@@ -8827,7 +8827,7 @@
         <f>AH61+AI61+AJ61</f>
       </c>
       <c r="AM61" s="5">
-        <v>187867.951225735</v>
+        <v>167645.08566528815</v>
       </c>
       <c r="AN61" s="6">
         <f>AL61-AM61</f>
@@ -9181,13 +9181,13 @@
         <f>$B$4</f>
       </c>
       <c r="H31" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I31" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J31" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K31" s="4">
         <f>D31*H31</f>
@@ -9274,7 +9274,7 @@
         <f>AH31+AI31+AJ31</f>
       </c>
       <c r="AM31" s="5">
-        <v>265657.78890706116</v>
+        <v>265536.875</v>
       </c>
       <c r="AN31" s="6">
         <f>AL31-AM31</f>
@@ -9303,13 +9303,13 @@
         <f>AK31</f>
       </c>
       <c r="H32" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I32" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J32" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K32" s="4">
         <f>D32*H32</f>
@@ -9396,7 +9396,7 @@
         <f>AH32+AI32+AJ32</f>
       </c>
       <c r="AM32" s="5">
-        <v>282034.18679049064</v>
+        <v>281778.4505456331</v>
       </c>
       <c r="AN32" s="6">
         <f>AL32-AM32</f>
@@ -9425,13 +9425,13 @@
         <f>AK32</f>
       </c>
       <c r="H33" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I33" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J33" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K33" s="4">
         <f>D33*H33</f>
@@ -9518,7 +9518,7 @@
         <f>AH33+AI33+AJ33</f>
       </c>
       <c r="AM33" s="5">
-        <v>299160.0214776577</v>
+        <v>298754.4861960199</v>
       </c>
       <c r="AN33" s="6">
         <f>AL33-AM33</f>
@@ -9547,13 +9547,13 @@
         <f>AK33</f>
       </c>
       <c r="H34" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I34" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J34" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K34" s="4">
         <f>D34*H34</f>
@@ -9640,7 +9640,7 @@
         <f>AH34+AI34+AJ34</f>
       </c>
       <c r="AM34" s="5">
-        <v>317067.4185265041</v>
+        <v>316495.9706220479</v>
       </c>
       <c r="AN34" s="6">
         <f>AL34-AM34</f>
@@ -9669,13 +9669,13 @@
         <f>AK34</f>
       </c>
       <c r="H35" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I35" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J35" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K35" s="4">
         <f>D35*H35</f>
@@ -9762,7 +9762,7 @@
         <f>AH35+AI35+AJ35</f>
       </c>
       <c r="AM35" s="5">
-        <v>335789.8556932355</v>
+        <v>335035.1720944865</v>
       </c>
       <c r="AN35" s="6">
         <f>AL35-AM35</f>
@@ -9791,13 +9791,13 @@
         <f>AK35</f>
       </c>
       <c r="H36" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I36" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J36" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K36" s="4">
         <f>D36*H36</f>
@@ -9884,7 +9884,7 @@
         <f>AH36+AI36+AJ36</f>
       </c>
       <c r="AM36" s="5">
-        <v>355362.21966919454</v>
+        <v>354405.6910277569</v>
       </c>
       <c r="AN36" s="6">
         <f>AL36-AM36</f>
@@ -9913,13 +9913,13 @@
         <f>AK36</f>
       </c>
       <c r="H37" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I37" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J37" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K37" s="4">
         <f>D37*H37</f>
@@ -10006,7 +10006,7 @@
         <f>AH37+AI37+AJ37</f>
       </c>
       <c r="AM37" s="5">
-        <v>375820.86518242897</v>
+        <v>374642.5146638829</v>
       </c>
       <c r="AN37" s="6">
         <f>AL37-AM37</f>
@@ -10035,13 +10035,13 @@
         <f>AK37</f>
       </c>
       <c r="H38" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I38" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J38" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K38" s="4">
         <f>D38*H38</f>
@@ -10128,7 +10128,7 @@
         <f>AH38+AI38+AJ38</f>
       </c>
       <c r="AM38" s="5">
-        <v>397203.6765632718</v>
+        <v>395782.07398441964</v>
       </c>
       <c r="AN38" s="6">
         <f>AL38-AM38</f>
@@ -10157,13 +10157,13 @@
         <f>AK38</f>
       </c>
       <c r="H39" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I39" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J39" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K39" s="4">
         <f>D39*H39</f>
@@ -10250,7 +10250,7 @@
         <f>AH39+AI39+AJ39</f>
       </c>
       <c r="AM39" s="5">
-        <v>419550.13187723135</v>
+        <v>417862.3029415951</v>
       </c>
       <c r="AN39" s="6">
         <f>AL39-AM39</f>
@@ -10279,13 +10279,13 @@
         <f>AK39</f>
       </c>
       <c r="H40" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I40" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J40" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K40" s="4">
         <f>D40*H40</f>
@@ -10372,7 +10372,7 @@
         <f>AH40+AI40+AJ40</f>
       </c>
       <c r="AM40" s="5">
-        <v>442901.36973266513</v>
+        <v>440922.7001034902</v>
       </c>
       <c r="AN40" s="6">
         <f>AL40-AM40</f>
@@ -10401,13 +10401,13 @@
         <f>AK40</f>
       </c>
       <c r="H41" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I41" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J41" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K41" s="4">
         <f>D41*H41</f>
@@ -10494,7 +10494,7 @@
         <f>AH41+AI41+AJ41</f>
       </c>
       <c r="AM41" s="5">
-        <v>436398.66163337044</v>
+        <v>434102.79557013465</v>
       </c>
       <c r="AN41" s="6">
         <f>AL41-AM41</f>
@@ -10523,13 +10523,13 @@
         <f>AK41</f>
       </c>
       <c r="H42" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I42" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J42" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K42" s="4">
         <f>D42*H42</f>
@@ -10616,7 +10616,7 @@
         <f>AH42+AI42+AJ42</f>
       </c>
       <c r="AM42" s="5">
-        <v>430082.0202540468</v>
+        <v>427448.6797764319</v>
       </c>
       <c r="AN42" s="6">
         <f>AL42-AM42</f>
@@ -10645,13 +10645,13 @@
         <f>AK42</f>
       </c>
       <c r="H43" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I43" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J43" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K43" s="4">
         <f>D43*H43</f>
@@ -10738,7 +10738,7 @@
         <f>AH43+AI43+AJ43</f>
       </c>
       <c r="AM43" s="5">
-        <v>423961.6170362026</v>
+        <v>420969.44158255693</v>
       </c>
       <c r="AN43" s="6">
         <f>AL43-AM43</f>
@@ -10767,13 +10767,13 @@
         <f>AK43</f>
       </c>
       <c r="H44" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I44" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J44" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K44" s="4">
         <f>D44*H44</f>
@@ -10860,7 +10860,7 @@
         <f>AH44+AI44+AJ44</f>
       </c>
       <c r="AM44" s="5">
-        <v>418047.725727001</v>
+        <v>414674.2390725757</v>
       </c>
       <c r="AN44" s="6">
         <f>AL44-AM44</f>
@@ -10889,13 +10889,13 @@
         <f>AK44</f>
       </c>
       <c r="H45" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I45" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J45" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K45" s="4">
         <f>D45*H45</f>
@@ -10982,7 +10982,7 @@
         <f>AH45+AI45+AJ45</f>
       </c>
       <c r="AM45" s="5">
-        <v>412350.69843896537</v>
+        <v>408572.27555707115</v>
       </c>
       <c r="AN45" s="6">
         <f>AL45-AM45</f>
@@ -11011,13 +11011,13 @@
         <f>AK45</f>
       </c>
       <c r="H46" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I46" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J46" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K46" s="4">
         <f>D46*H46</f>
@@ -11104,7 +11104,7 @@
         <f>AH46+AI46+AJ46</f>
       </c>
       <c r="AM46" s="5">
-        <v>406880.94090200716</v>
+        <v>402672.7745604222</v>
       </c>
       <c r="AN46" s="6">
         <f>AL46-AM46</f>
@@ -11133,13 +11133,13 @@
         <f>AK46</f>
       </c>
       <c r="H47" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I47" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J47" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K47" s="4">
         <f>D47*H47</f>
@@ -11226,7 +11226,7 @@
         <f>AH47+AI47+AJ47</f>
       </c>
       <c r="AM47" s="5">
-        <v>401648.88729501504</v>
+        <v>396984.9541107418</v>
       </c>
       <c r="AN47" s="6">
         <f>AL47-AM47</f>
@@ -11255,13 +11255,13 @@
         <f>AK47</f>
       </c>
       <c r="H48" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I48" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J48" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K48" s="4">
         <f>D48*H48</f>
@@ -11348,7 +11348,7 @@
         <f>AH48+AI48+AJ48</f>
       </c>
       <c r="AM48" s="5">
-        <v>396395.2714553727</v>
+        <v>391260.51067077345</v>
       </c>
       <c r="AN48" s="6">
         <f>AL48-AM48</f>
@@ -11377,13 +11377,13 @@
         <f>AK48</f>
       </c>
       <c r="H49" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I49" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J49" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K49" s="4">
         <f>D49*H49</f>
@@ -11470,7 +11470,7 @@
         <f>AH49+AI49+AJ49</f>
       </c>
       <c r="AM49" s="5">
-        <v>391025.3714186273</v>
+        <v>385404.9190490516</v>
       </c>
       <c r="AN49" s="6">
         <f>AL49-AM49</f>
@@ -11499,13 +11499,13 @@
         <f>AK49</f>
       </c>
       <c r="H50" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I50" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J50" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K50" s="4">
         <f>D50*H50</f>
@@ -11592,7 +11592,7 @@
         <f>AH50+AI50+AJ50</f>
       </c>
       <c r="AM50" s="5">
-        <v>385534.03824671044</v>
+        <v>379412.680707981</v>
       </c>
       <c r="AN50" s="6">
         <f>AL50-AM50</f>
@@ -11621,13 +11621,13 @@
         <f>AK50</f>
       </c>
       <c r="H51" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I51" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J51" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K51" s="4">
         <f>D51*H51</f>
@@ -11714,7 +11714,7 @@
         <f>AH51+AI51+AJ51</f>
       </c>
       <c r="AM51" s="5">
-        <v>379915.9008719914</v>
+        <v>373278.0686892691</v>
       </c>
       <c r="AN51" s="6">
         <f>AL51-AM51</f>
@@ -11743,13 +11743,13 @@
         <f>AK51</f>
       </c>
       <c r="H52" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I52" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J52" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K52" s="4">
         <f>D52*H52</f>
@@ -11836,7 +11836,7 @@
         <f>AH52+AI52+AJ52</f>
       </c>
       <c r="AM52" s="5">
-        <v>374165.35758135846</v>
+        <v>366995.11900361395</v>
       </c>
       <c r="AN52" s="6">
         <f>AL52-AM52</f>
@@ -11865,13 +11865,13 @@
         <f>AK52</f>
       </c>
       <c r="H53" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I53" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J53" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K53" s="4">
         <f>D53*H53</f>
@@ -11958,7 +11958,7 @@
         <f>AH53+AI53+AJ53</f>
       </c>
       <c r="AM53" s="5">
-        <v>368276.56716195564</v>
+        <v>360557.621686716</v>
       </c>
       <c r="AN53" s="6">
         <f>AL53-AM53</f>
@@ -11987,13 +11987,13 @@
         <f>AK53</f>
       </c>
       <c r="H54" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I54" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J54" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K54" s="4">
         <f>D54*H54</f>
@@ -12080,7 +12080,7 @@
         <f>AH54+AI54+AJ54</f>
       </c>
       <c r="AM54" s="5">
-        <v>362243.4396937175</v>
+        <v>353959.1115075578</v>
       </c>
       <c r="AN54" s="6">
         <f>AL54-AM54</f>
@@ -12109,13 +12109,13 @@
         <f>AK54</f>
       </c>
       <c r="H55" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I55" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J55" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K55" s="4">
         <f>D55*H55</f>
@@ -12202,7 +12202,7 @@
         <f>AH55+AI55+AJ55</f>
       </c>
       <c r="AM55" s="5">
-        <v>356059.6269732234</v>
+        <v>347192.85831432755</v>
       </c>
       <c r="AN55" s="6">
         <f>AL55-AM55</f>
@@ -12231,13 +12231,13 @@
         <f>AK55</f>
       </c>
       <c r="H56" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I56" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J56" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K56" s="4">
         <f>D56*H56</f>
@@ -12324,7 +12324,7 @@
         <f>AH56+AI56+AJ56</f>
       </c>
       <c r="AM56" s="5">
-        <v>349718.51255275356</v>
+        <v>340251.85700276913</v>
       </c>
       <c r="AN56" s="6">
         <f>AL56-AM56</f>
@@ -12353,13 +12353,13 @@
         <f>AK56</f>
       </c>
       <c r="H57" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I57" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J57" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K57" s="4">
         <f>D57*H57</f>
@@ -12446,7 +12446,7 @@
         <f>AH57+AI57+AJ57</f>
       </c>
       <c r="AM57" s="5">
-        <v>343213.20137776446</v>
+        <v>333128.8170911341</v>
       </c>
       <c r="AN57" s="6">
         <f>AL57-AM57</f>
@@ -12475,13 +12475,13 @@
         <f>AK57</f>
       </c>
       <c r="H58" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I58" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J58" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K58" s="4">
         <f>D58*H58</f>
@@ -12568,7 +12568,7 @@
         <f>AH58+AI58+AJ58</f>
       </c>
       <c r="AM58" s="5">
-        <v>336536.50900531595</v>
+        <v>325816.1518852734</v>
       </c>
       <c r="AN58" s="6">
         <f>AL58-AM58</f>
@@ -12597,13 +12597,13 @@
         <f>AK58</f>
       </c>
       <c r="H59" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I59" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J59" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K59" s="4">
         <f>D59*H59</f>
@@ -12690,7 +12690,7 @@
         <f>AH59+AI59+AJ59</f>
       </c>
       <c r="AM59" s="5">
-        <v>329680.95038526563</v>
+        <v>318305.9672167547</v>
       </c>
       <c r="AN59" s="6">
         <f>AL59-AM59</f>
@@ -12719,13 +12719,13 @@
         <f>AK59</f>
       </c>
       <c r="H60" s="15">
-        <f>EXP($B$8-$B$9)-1</f>
+        <f>$B$8-$B$9</f>
       </c>
       <c r="I60" s="15">
-        <f>EXP($B$10-$B$11)-1</f>
+        <f>$B$10-$B$11</f>
       </c>
       <c r="J60" s="15">
-        <f>EXP($B$12-$B$13)-1</f>
+        <f>$B$12-$B$13</f>
       </c>
       <c r="K60" s="4">
         <f>D60*H60</f>
@@ -12812,7 +12812,7 @@
         <f>AH60+AI60+AJ60</f>
       </c>
       <c r="AM60" s="5">
-        <v>322638.7281853139</v>
+        <v>310590.049736207</v>
       </c>
       <c r="AN60" s="6">
         <f>AL60-AM60</f>

</xml_diff>